<commit_message>
Update AI Audit Log_DangThanhTung.xlsx
</commit_message>
<xml_diff>
--- a/AI Audit Log_DangThanhTung.xlsx
+++ b/AI Audit Log_DangThanhTung.xlsx
@@ -4,18 +4,17 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12885" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12885"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
-    <sheet name="Week1" sheetId="2" r:id="rId2"/>
-    <sheet name="Week2" sheetId="3" r:id="rId3"/>
-    <sheet name="Week3" sheetId="4" r:id="rId4"/>
-    <sheet name="Week4" sheetId="5" r:id="rId5"/>
-    <sheet name="Week5" sheetId="6" r:id="rId6"/>
-    <sheet name="Week6" sheetId="7" r:id="rId7"/>
-    <sheet name="Week7" sheetId="8" r:id="rId8"/>
-    <sheet name="Week8" sheetId="9" r:id="rId9"/>
+    <sheet name="Week2" sheetId="2" r:id="rId2"/>
+    <sheet name="Week3" sheetId="3" r:id="rId3"/>
+    <sheet name="Week4" sheetId="4" r:id="rId4"/>
+    <sheet name="Week5" sheetId="5" r:id="rId5"/>
+    <sheet name="Week6" sheetId="6" r:id="rId6"/>
+    <sheet name="Week7" sheetId="7" r:id="rId7"/>
+    <sheet name="Week8" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="71">
   <si>
     <t>STT</t>
   </si>
@@ -174,6 +173,81 @@
   </si>
   <si>
     <t>AI đề xuất tách frontend, backend, database, testing. Sau khi đánh giá, quyết định phân chia theo năng lực thực tế từng thành viên thay vì chia đều, giúp tối ưu tốc độ hoàn thành và giảm conflict khi merge code.</t>
+  </si>
+  <si>
+    <t>Giai đoạn</t>
+  </si>
+  <si>
+    <t>Nội dung</t>
+  </si>
+  <si>
+    <t>Phản hồi AI</t>
+  </si>
+  <si>
+    <t>Phản hồi Con người</t>
+  </si>
+  <si>
+    <t>Khác biệt</t>
+  </si>
+  <si>
+    <t>Sequence Diagram</t>
+  </si>
+  <si>
+    <t>Vẽ diagram Car Return process</t>
+  </si>
+  <si>
+    <t>Vẽ đúng UML, đủ các actor như BookingController, BookingService, CarRepository, BookingRepository, PaymentService. Tuy nhiên vẫn tập trung vào luồng chính nên chưa xử lý tốt các tình huống phát sinh như thanh toán thất bại hay tranh chấp khi xác nhận booking.</t>
+  </si>
+  <si>
+    <t>Bổ sung đầy đủ các nhánh xử lý như thanh toán thành công / thất bại, thêm cơ chế retry khi cần và xử lý khóa giao dịch khi có nhiều request đồng thời. Ngoài ra còn tính luôn các case như timeout hoặc lỗi inventory.</t>
+  </si>
+  <si>
+    <t>AI đi nhanh theo luồng chính nên gọn nhưng thiếu chiều sâu. Con người làm chậm hơn nhưng bao quát được các tình huống thực tế và tính ổn định hệ thống.</t>
+  </si>
+  <si>
+    <t>Activity Diagram</t>
+  </si>
+  <si>
+    <t>Vẽ Car Return + Inspection + Fee Calculation</t>
+  </si>
+  <si>
+    <t>Trình bày các bước rõ ràng theo trình tự, có decision cho việc phát sinh phí. Tuy nhiên các bước bị xếp tuần tự nên chưa tối ưu, thiếu điều kiện ràng buộc và chưa phản ánh đúng logic nghiệp vụ thực tế.</t>
+  </si>
+  <si>
+    <t>Tách các bước có thể chạy song song như kiểm tra xe và tính phí, thêm điều kiện ràng buộc rõ ràng, đồng thời bổ sung luồng xử lý khi xe bị hư hỏng dẫn đến cập nhật trạng thái không khả dụng.</t>
+  </si>
+  <si>
+    <t>AI tập trung vào flow dễ hiểu, còn con người tối ưu lại quy trình để sát thực tế hơn và cải thiện hiệu suất xử lý.</t>
+  </si>
+  <si>
+    <t>Class Diagram</t>
+  </si>
+  <si>
+    <t>Tạo class cho User, Staff, Customer, Booking, Car, Payment, Repositories</t>
+  </si>
+  <si>
+    <t>Định nghĩa đúng các entity cơ bản nhưng còn đơn giản, dùng kiểu dữ liệu chung chung như String cho status, thiếu constraint cho amount và chưa rõ quan hệ giữa các class. Một số hàm nghiệp vụ quan trọng cũng chưa được thể hiện.</t>
+  </si>
+  <si>
+    <t>Chuẩn hóa lại bằng enum cho status, thêm ràng buộc dữ liệu rõ ràng, làm rõ quan hệ 1-n giữa Customer và Booking, đồng thời bổ sung các method nghiệp vụ như tính phí trễ, kiểm tra khả dụng xe và hoàn tiền.</t>
+  </si>
+  <si>
+    <t>AI thiên về khung tổng quát, Con người đi sâu vào business logic và thiết kế chặt chẽ hơn.</t>
+  </si>
+  <si>
+    <t>Design Quality</t>
+  </si>
+  <si>
+    <t>So sánh tổng thể AI vs Con người</t>
+  </si>
+  <si>
+    <t>Tổng thể đúng chuẩn UML, dựng nhanh và rõ ràng, phù hợp để phác thảo ban đầu. Tuy nhiên còn thiếu ngữ cảnh nghiệp vụ, chưa xử lý hết edge case và chưa tối ưu hiệu suất hệ thống.</t>
+  </si>
+  <si>
+    <t>Thiết kế đầy đủ hơn với logic nghiệp vụ rõ ràng, xử lý tốt các tình huống lỗi, tối ưu luồng xử lý song song và bao quát các trường hợp đặc biệt như timeout hay hư hỏng xe.</t>
+  </si>
+  <si>
+    <t>AI mạnh ở tốc độ và khung ban đầu, Con người mạnh ở chiều sâu thiết kế, tính thực tế và độ hoàn thiện hệ thống.</t>
   </si>
   <si>
     <t>W</t>
@@ -828,12 +902,24 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -850,9 +936,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1203,73 +1286,73 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" spans="1:5">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4"/>
-    </row>
-    <row r="2" ht="71.25" spans="1:4">
-      <c r="A2" s="5">
+      <c r="E1" s="8"/>
+    </row>
+    <row r="2" ht="57" spans="1:4">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" ht="57" spans="1:4">
-      <c r="A3" s="5">
+      <c r="A3" s="9">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" ht="71.25" spans="1:4">
-      <c r="A4" s="5">
+      <c r="A4" s="9">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" ht="85.5" spans="1:4">
-      <c r="A5" s="5">
+    <row r="5" ht="71.25" spans="1:4">
+      <c r="A5" s="9">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="6" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1291,128 +1374,128 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" spans="1:4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" ht="71.25" spans="1:4">
-      <c r="A2" s="2" t="s">
+    <row r="2" ht="57" spans="1:4">
+      <c r="A2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" ht="57" spans="1:4">
-      <c r="A3" s="2" t="s">
+    <row r="3" ht="42.75" spans="1:4">
+      <c r="A3" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" ht="57" spans="1:4">
-      <c r="A4" s="2" t="s">
+    <row r="4" ht="42.75" spans="1:4">
+      <c r="A4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" ht="57" spans="1:4">
-      <c r="A5" s="2" t="s">
+    <row r="5" ht="42.75" spans="1:4">
+      <c r="A5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="6" ht="42.75" spans="1:4">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" ht="42.75" spans="1:4">
-      <c r="A7" s="2" t="s">
+    <row r="7" ht="28.5" spans="1:4">
+      <c r="A7" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" ht="42.75" spans="1:4">
-      <c r="A8" s="2" t="s">
+    <row r="8" ht="28.5" spans="1:4">
+      <c r="A8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="9" ht="42.75" spans="1:4">
-      <c r="A9" s="2" t="s">
+    <row r="9" ht="28.5" spans="1:4">
+      <c r="A9" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="6" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1425,9 +1508,118 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
-  <sheetData/>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="4" outlineLevelCol="5"/>
+  <cols>
+    <col min="1" max="1" width="4.375" customWidth="1"/>
+    <col min="2" max="2" width="16.375" customWidth="1"/>
+    <col min="3" max="3" width="17.125" customWidth="1"/>
+    <col min="4" max="4" width="57.375" customWidth="1"/>
+    <col min="5" max="5" width="47" customWidth="1"/>
+    <col min="6" max="6" width="54.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" ht="57" spans="1:6">
+      <c r="A2" s="2">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" ht="57" spans="1:6">
+      <c r="A3" s="2">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" ht="71.25" spans="1:6">
+      <c r="A4" s="2">
+        <v>7</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" ht="57" spans="1:6">
+      <c r="A5" s="2">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
@@ -1452,7 +1644,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1492,15 +1684,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
 </file>
</xml_diff>